<commit_message>
Update checklist, Word plan, and Excel finance sheet to match Vang My restaurant and pilot event parameters
</commit_message>
<xml_diff>
--- a/Plan/Tram Hen Ho Hai Phong - Bai toan tai chinh.xlsx
+++ b/Plan/Tram Hen Ho Hai Phong - Bai toan tai chinh.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bài toán 30 khách" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bài toán 20 khách" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bài toán 20 khách (Pilot)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bài toán 30 khách" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="So sánh hiệu quả" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -545,8 +545,8 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="49" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="76" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
@@ -554,7 +554,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỰ TOÁN DOANH THU &amp; CHI PHÍ - QUY MÔ 30 KHÁCH</t>
+          <t>DỰ TOÁN DOANH THU &amp; CHI PHÍ - QUY MÔ 20 KHÁCH (ĐỐI TÁC NHÀ HÀNG VANG MY)</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Đơn giá mỗi vé tham gia</t>
+          <t>Đơn giá mỗi vé tham gia (Thanh toán trước)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
@@ -605,11 +605,11 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tổng số khách (15 Nam &amp; 15 Nữ)</t>
+          <t>Tổng số khách chốt chính thức (10 Nam &amp; 10 Nữ)</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D5" s="7" t="n"/>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>30 khách x Giá vé</t>
+          <t>20 khách x Giá vé (Chuyển khoản vào STK BTC)</t>
         </is>
       </c>
       <c r="C6" s="9">
@@ -637,12 +637,12 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Chi phí F&amp;B (Nước + Teabreak)</t>
+          <t>Chi phí F&amp;B tại Vang My Restaurant</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>30 phần x 80.000 VNĐ</t>
+          <t>20 phần nước uống + teabreak x 80.000 VNĐ</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -662,7 +662,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>30 phần x 40.000 VNĐ</t>
+          <t>20 phần quà tặng hậu event x 40.000 VNĐ</t>
         </is>
       </c>
       <c r="C9" s="14">
@@ -682,32 +682,32 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Bản in màu + Bút viết</t>
+          <t>Match Card, Prompt Card bản in màu + Bút</t>
         </is>
       </c>
       <c r="C10" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Thuê địa điểm (Lounge/Cafe VIP)</t>
+          <t>Thuê địa điểm (Nhà hàng Vang My)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Gói bao trọn khu vực riêng (3 giờ)</t>
+          <t>Bao trọn gói khu vực riêng biệt tổ chức</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>2500000</v>
+        <v>2000000</v>
       </c>
     </row>
     <row r="12">
@@ -718,7 +718,7 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Nhân sự chuyên nghiệp</t>
+          <t>Thuê MC dẫn dắt chính theo kịch bản</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
@@ -731,19 +731,19 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Marketing &amp; Lọc hồ sơ</t>
+          <t>Marketing tuyển sinh (Zalo/Facebook)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Chạy quảng cáo Facebook Ads + Telesale</t>
+          <t>Chi phí quảng cáo thu hút hồ sơ đầu vào</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>2500000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="14">
@@ -754,14 +754,14 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>2 bạn hỗ trợ check-in, xoay bàn</t>
+          <t>1 nhân sự check-in kiêm hỗ trợ MC xoay bàn</t>
         </is>
       </c>
       <c r="C14" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>600000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="15">
@@ -772,7 +772,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Chi phí Biến đổi + Cố định</t>
+          <t>Chi phí Biến đổi + Chi phí Cố định</t>
         </is>
       </c>
       <c r="C15" s="18" t="n"/>
@@ -838,7 +838,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DỰ TOÁN DOANH THU &amp; CHI PHÍ - QUY MÔ 20 KHÁCH</t>
+          <t>DỰ TOÁN DOANH THU &amp; CHI PHÍ - QUY MÔ 30 KHÁCH</t>
         </is>
       </c>
     </row>
@@ -889,11 +889,11 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tổng số khách (10 Nam &amp; 10 Nữ)</t>
+          <t>Tổng số khách (15 Nam &amp; 15 Nữ)</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D5" s="7" t="n"/>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>20 khách x Giá vé</t>
+          <t>30 khách x Giá vé</t>
         </is>
       </c>
       <c r="C6" s="9">
@@ -926,7 +926,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>20 phần x 80.000 VNĐ</t>
+          <t>30 phần x 80.000 VNĐ</t>
         </is>
       </c>
       <c r="C8" s="12">
@@ -946,7 +946,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>20 phần x 40.000 VNĐ</t>
+          <t>30 phần x 40.000 VNĐ</t>
         </is>
       </c>
       <c r="C9" s="14">
@@ -973,25 +973,25 @@
         <v>1</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Thuê địa điểm (Phòng VIP/Lounge nhỏ)</t>
+          <t>Thuê địa điểm (Lounge/Cafe VIP)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Bao trọn khu vực riêng quy mô 20 người</t>
+          <t>Gói bao trọn khu vực riêng (3 giờ)</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>2000000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="12">
@@ -1020,14 +1020,14 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Chi phí quảng cáo &amp; telesale chọn lọc</t>
+          <t>Chạy quảng cáo Facebook Ads + Telesale</t>
         </is>
       </c>
       <c r="C13" s="14" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>1800000</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="14">
@@ -1038,14 +1038,14 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>1 bạn hỗ trợ check-in, xoay bàn</t>
+          <t>2 bạn hỗ trợ check-in, xoay bàn</t>
         </is>
       </c>
       <c r="C14" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>300000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="15">
@@ -1115,10 +1115,10 @@
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="77" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1171,19 +1171,19 @@
         <v>499000</v>
       </c>
       <c r="C4" s="13">
-        <f>'Bài toán 20 khách'!D6</f>
+        <f>'Bài toán 20 khách (Pilot)'!D6</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>'Bài toán 20 khách'!D15</f>
+        <f>'Bài toán 20 khách (Pilot)'!D15</f>
         <v/>
       </c>
       <c r="E4" s="23">
-        <f>'Bài toán 20 khách'!D16</f>
+        <f>'Bài toán 20 khách (Pilot)'!D16</f>
         <v/>
       </c>
       <c r="F4" s="24">
-        <f>'Bài toán 20 khách'!D17</f>
+        <f>'Bài toán 20 khách (Pilot)'!D17</f>
         <v/>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         <v/>
       </c>
       <c r="D5" s="15">
-        <f>2000*20 + 1000*20 + 200000 + 2000000 + 1200000 + 1800000 + 300000</f>
+        <f>2000000 + 1200000 + 1800000 + 300000 + 200000 + (100000*20) + (50000*20)</f>
         <v/>
       </c>
       <c r="E5" s="26">
@@ -1253,7 +1253,7 @@
         <v/>
       </c>
       <c r="D7" s="15">
-        <f>3000*30 + 1500*30 + 300000 + 2500000 + 1200000 + 2500000 + 600000</f>
+        <f>2500000 + 1200000 + 2500000 + 600000 + 300000 + (100000*30) + (50000*30)</f>
         <v/>
       </c>
       <c r="E7" s="26">

</xml_diff>